<commit_message>
Update assignment description for KNN exercise to specify data standardization requirement
</commit_message>
<xml_diff>
--- a/KNN練習題/KNN-作業2.xlsx
+++ b/KNN練習題/KNN-作業2.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\1.教學\113-1資料探勘DataMining\KNN練習題\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\1.教學\3.資料探勘DataMining\Data Mining MarkDown\KNN練習題\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9720" tabRatio="720" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9720" tabRatio="720"/>
   </bookViews>
   <sheets>
     <sheet name="1.去年的資料(拿來訓練我們的Model)" sheetId="1" r:id="rId1"/>
-    <sheet name="2.以KNN-單純算距離方式來驗證此Model正確性是否OK" sheetId="2" r:id="rId2"/>
-    <sheet name="3.課本原來的方法-有權重-影響距離半徑-非線性的指數" sheetId="3" r:id="rId3"/>
+    <sheet name="2.以KNN-單純算距離方式來驗證此Model正確性" sheetId="2" r:id="rId2"/>
+    <sheet name="3.加入權重" sheetId="4" r:id="rId3"/>
+    <sheet name="4.有權重-距離轉換成相似度(非線性的指數)-影響距離半徑" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>No</t>
   </si>
@@ -51,12 +52,20 @@
     <t>參加Tour</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
+  <si>
+    <t>題目說明: 去年共有20筆本旅行社回收問卷/及最後出團資料. 訓練模型前資料需先作標準化</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>以12筆資料作為已知, 以8筆資料作為驗證. 求出最佳的 : 誤差均方根及誤判率</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -94,8 +103,24 @@
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="新細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -120,6 +145,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0000FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -138,7 +175,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -171,6 +208,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -179,6 +234,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0000FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -453,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="16.2"/>
   <cols>
     <col min="1" max="3" width="8.88671875" style="1"/>
@@ -461,90 +521,84 @@
     <col min="10" max="10" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:14">
+      <c r="A1" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="15"/>
+      <c r="B2" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="15"/>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="1" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-    </row>
-    <row r="3" spans="1:10" s="1" customFormat="1">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+    </row>
+    <row r="5" spans="1:14" s="1" customFormat="1">
+      <c r="A5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="I3" s="8" t="s">
+      <c r="H5" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="1">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2">
+    <row r="6" spans="1:14">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2">
         <v>58</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C6" s="2">
         <v>9</v>
-      </c>
-      <c r="D4" s="3">
-        <v>1</v>
-      </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="1">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2">
-        <v>30</v>
-      </c>
-      <c r="C5" s="2">
-        <v>6</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2">
-        <v>37</v>
-      </c>
-      <c r="C6" s="2">
-        <v>12</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -555,15 +609,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:14">
       <c r="A7" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B7" s="2">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3">
         <v>0</v>
@@ -574,34 +628,34 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:14">
       <c r="A8" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B8" s="2">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C8" s="2">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
       <c r="J8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B9" s="2">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="C9" s="2">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D9" s="3">
         <v>0</v>
@@ -612,53 +666,53 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:14">
       <c r="A10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B10" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
       <c r="J10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B11" s="2">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="C11" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
       <c r="J11" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B12" s="2">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D12" s="3">
         <v>1</v>
@@ -669,15 +723,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:14">
       <c r="A13" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B13" s="2">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C13" s="2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D13" s="3">
         <v>1</v>
@@ -688,53 +742,53 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:14">
       <c r="A14" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B14" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="2">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D14" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
       <c r="J14" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B15" s="2">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
       <c r="J15" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" s="2">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="C16" s="2">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D16" s="3">
         <v>0</v>
@@ -747,13 +801,13 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B17" s="2">
         <v>18</v>
       </c>
       <c r="C17" s="2">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D17" s="3">
         <v>0</v>
@@ -766,13 +820,13 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B18" s="2">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="C18" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="3">
         <v>0</v>
@@ -785,51 +839,51 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B19" s="2">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="C19" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D19" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" s="9"/>
       <c r="I19" s="9"/>
       <c r="J19" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B20" s="2">
-        <v>46</v>
+        <v>71</v>
       </c>
       <c r="C20" s="2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D20" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
       <c r="J20" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="1">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B21" s="2">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C21" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D21" s="3">
         <v>1</v>
@@ -842,70 +896,70 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="1">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B22" s="2">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C22" s="2">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="1">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B23" s="2">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="C23" s="2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="1">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B24" s="2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C24" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D24" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
       <c r="J24" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="1">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B25" s="2">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C25" s="2">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D25" s="3">
         <v>0</v>
@@ -913,6 +967,44 @@
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
       <c r="J25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="1">
+        <v>21</v>
+      </c>
+      <c r="B26" s="2">
+        <v>47</v>
+      </c>
+      <c r="C26" s="2">
+        <v>10</v>
+      </c>
+      <c r="D26" s="3">
+        <v>1</v>
+      </c>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="1">
+        <v>22</v>
+      </c>
+      <c r="B27" s="2">
+        <v>36</v>
+      </c>
+      <c r="C27" s="2">
+        <v>18</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="1">
         <v>0</v>
       </c>
     </row>
@@ -925,6 +1017,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="16.2"/>
   <sheetData/>
@@ -935,6 +1030,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.2"/>
+  <sheetData/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="16.2"/>
   <sheetData/>

</xml_diff>